<commit_message>
test(e2e): add e2e test for article deletion
Refs: #11
</commit_message>
<xml_diff>
--- a/docs/coverages.xlsx
+++ b/docs/coverages.xlsx
@@ -255,13 +255,13 @@
             <v>0.75</v>
           </cell>
           <cell r="C6">
-            <v>0.605769230769231</v>
+            <v>0.855769230769231</v>
           </cell>
           <cell r="D6">
-            <v>0.152777777777778</v>
+            <v>0.652777777777778</v>
           </cell>
           <cell r="E6">
-            <v>0.502849002849003</v>
+            <v>0.752849002849003</v>
           </cell>
         </row>
       </sheetData>
@@ -280,7 +280,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q40"/>
-  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22.51"/>
@@ -359,13 +359,13 @@
       </c>
       <c r="C3" s="3" t="n">
         <f aca="false" t="array" ref="C3:E3">[2]Summary!C6:E6</f>
-        <v>0.605769230769231</v>
+        <v>0.855769230769231</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.152777777777778</v>
+        <v>0.652777777777778</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.502849002849003</v>
+        <v>0.752849002849003</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
[#11] Add e2e test for article deletion (#31)
* test(e2e): add e2e test for article deletion

Refs: #11

* fix(e2e): correct broken article editor & details url regex

Refs: #11

* chore(config): set headless mode based on CI environment

Refs: #11

* fix(e2e): enable headless mode for article deletion tests

Refs: #11

* refactor(e2e): format spacing in ARTICLE_EDITOR regex function

Refs: #11

* fix(config): correct headless mode configuration in Playwright setup

Refs: #11

* fix(e2e): await deleteArticleButton click in deleteArticle method

Refs: #11

* fix(e2e): remove unused parameters in concurrent update test for articles

Refs: #11

* fix(e2e): streamline article update process by using updateArticle method

Refs: #11

---------

Co-authored-by: idembele70 <idembele70@gmail>
</commit_message>
<xml_diff>
--- a/docs/coverages.xlsx
+++ b/docs/coverages.xlsx
@@ -255,13 +255,13 @@
             <v>0.75</v>
           </cell>
           <cell r="C6">
-            <v>0.605769230769231</v>
+            <v>0.855769230769231</v>
           </cell>
           <cell r="D6">
-            <v>0.152777777777778</v>
+            <v>0.652777777777778</v>
           </cell>
           <cell r="E6">
-            <v>0.502849002849003</v>
+            <v>0.752849002849003</v>
           </cell>
         </row>
       </sheetData>
@@ -280,7 +280,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q40"/>
-  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22.51"/>
@@ -359,13 +359,13 @@
       </c>
       <c r="C3" s="3" t="n">
         <f aca="false" t="array" ref="C3:E3">[2]Summary!C6:E6</f>
-        <v>0.605769230769231</v>
+        <v>0.855769230769231</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.152777777777778</v>
+        <v>0.652777777777778</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.502849002849003</v>
+        <v>0.752849002849003</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>8</v>

</xml_diff>